<commit_message>
Data export W39-2026 (2026-09-27T06:18:28Z)
</commit_message>
<xml_diff>
--- a/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
+++ b/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
@@ -643,22 +643,22 @@
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>96529</v>
+        <v>99091</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>44.40095122882389</v>
+        <v>44.40655179367675</v>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>180652:00:00</t>
+          <t>185274:00:00</t>
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>180652</v>
+        <v>185274</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>44.79267654665057</v>
+        <v>44.65940317215446</v>
       </c>
     </row>
     <row r="3">
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>55483</v>
+        <v>56955</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>25.52080698058444</v>
+        <v>25.52376257590356</v>
       </c>
       <c r="E3" s="10" t="inlineStr"/>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>103907:00:00</t>
+          <t>107363:00:00</t>
         </is>
       </c>
       <c r="G3" s="10" t="n">
-        <v>103907</v>
+        <v>107363</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>25.7637482116601</v>
+        <v>25.87933278696428</v>
       </c>
     </row>
     <row r="4">
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>65391</v>
+        <v>67099</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>30.07824179059167</v>
+        <v>30.06968563041968</v>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>118748:00:00</t>
+          <t>122223:00:00</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>118748</v>
+        <v>122223</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>29.44357524168933</v>
+        <v>29.46126404088126</v>
       </c>
     </row>
   </sheetData>
@@ -1175,7 +1175,7 @@
         <v>2191</v>
       </c>
       <c r="AM2" s="9" t="n">
-        <v>0</v>
+        <v>2562</v>
       </c>
       <c r="AN2" s="9" t="n">
         <v>0</v>
@@ -1338,7 +1338,7 @@
         <v>1488</v>
       </c>
       <c r="AM3" s="10" t="n">
-        <v>0</v>
+        <v>1472</v>
       </c>
       <c r="AN3" s="10" t="n">
         <v>0</v>
@@ -1501,7 +1501,7 @@
         <v>1441</v>
       </c>
       <c r="AM4" s="11" t="n">
-        <v>0</v>
+        <v>1708</v>
       </c>
       <c r="AN4" s="11" t="n">
         <v>0</v>
@@ -1664,7 +1664,7 @@
         <v>5120</v>
       </c>
       <c r="AM5" s="12" t="n">
-        <v>0</v>
+        <v>5742</v>
       </c>
       <c r="AN5" s="12" t="n">
         <v>0</v>
@@ -2163,7 +2163,7 @@
         <v>3692</v>
       </c>
       <c r="AM2" s="9" t="n">
-        <v>0</v>
+        <v>4622</v>
       </c>
       <c r="AN2" s="9" t="n">
         <v>0</v>
@@ -2326,7 +2326,7 @@
         <v>2940</v>
       </c>
       <c r="AM3" s="10" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="AN3" s="10" t="n">
         <v>0</v>
@@ -2489,7 +2489,7 @@
         <v>2986</v>
       </c>
       <c r="AM4" s="11" t="n">
-        <v>0</v>
+        <v>3475</v>
       </c>
       <c r="AN4" s="11" t="n">
         <v>0</v>
@@ -2652,7 +2652,7 @@
         <v>9618</v>
       </c>
       <c r="AM5" s="12" t="n">
-        <v>0</v>
+        <v>11553</v>
       </c>
       <c r="AN5" s="12" t="n">
         <v>0</v>
@@ -3455,16 +3455,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>2562</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>1472</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1708</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>5742</v>
       </c>
     </row>
     <row r="40">
@@ -4491,16 +4491,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>4622</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>3475</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>11553</v>
       </c>
     </row>
     <row r="40">
@@ -5995,16 +5995,16 @@
         <v>5554</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>2562</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1472</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1708</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>5742</v>
       </c>
     </row>
     <row r="40">
@@ -6502,7 +6502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6962,6 +6962,18 @@
       <c r="B38" t="inlineStr">
         <is>
           <t>C:\TRC\trc_engine\outputs\weekly\Weekly W37-2026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>W38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>C:\TRC\trc_engine\outputs\weekly\Weekly W38-2026.xlsx</t>
         </is>
       </c>
     </row>
@@ -8327,7 +8339,7 @@
         <v>2191</v>
       </c>
       <c r="AN9" s="7" t="n">
-        <v>0</v>
+        <v>2562</v>
       </c>
       <c r="AO9" s="7" t="n">
         <v>0</v>
@@ -8495,7 +8507,7 @@
         <v>1488</v>
       </c>
       <c r="AN10" s="7" t="n">
-        <v>0</v>
+        <v>1472</v>
       </c>
       <c r="AO10" s="7" t="n">
         <v>0</v>
@@ -8663,7 +8675,7 @@
         <v>1441</v>
       </c>
       <c r="AN11" s="7" t="n">
-        <v>0</v>
+        <v>1708</v>
       </c>
       <c r="AO11" s="7" t="n">
         <v>0</v>
@@ -9163,7 +9175,7 @@
         <v>3692</v>
       </c>
       <c r="AN15" s="7" t="n">
-        <v>0</v>
+        <v>4622</v>
       </c>
       <c r="AO15" s="7" t="n">
         <v>0</v>
@@ -9331,7 +9343,7 @@
         <v>2940</v>
       </c>
       <c r="AN16" s="7" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="AO16" s="7" t="n">
         <v>0</v>
@@ -9499,7 +9511,7 @@
         <v>2986</v>
       </c>
       <c r="AN17" s="7" t="n">
-        <v>0</v>
+        <v>3475</v>
       </c>
       <c r="AO17" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Data export W39-2026 (2026-09-28T08:14:54Z)
</commit_message>
<xml_diff>
--- a/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
+++ b/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
@@ -643,22 +643,22 @@
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>99091</v>
+        <v>101379</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>44.40655179367675</v>
+        <v>44.40293277737872</v>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>185274:00:00</t>
+          <t>189238:00:00</t>
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>185274</v>
+        <v>189238</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>44.65940317215446</v>
+        <v>44.58197478278897</v>
       </c>
     </row>
     <row r="3">
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>56955</v>
+        <v>58397</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>25.52376257590356</v>
+        <v>25.57727009933601</v>
       </c>
       <c r="E3" s="10" t="inlineStr"/>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>107363:00:00</t>
+          <t>109949:00:00</t>
         </is>
       </c>
       <c r="G3" s="10" t="n">
-        <v>107363</v>
+        <v>109949</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>25.87933278696428</v>
+        <v>25.9025330292693</v>
       </c>
     </row>
     <row r="4">
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>67099</v>
+        <v>68540</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>30.06968563041968</v>
+        <v>30.01979712328527</v>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>122223:00:00</t>
+          <t>125285:00:00</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>122223</v>
+        <v>125285</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>29.46126404088126</v>
+        <v>29.51549218794173</v>
       </c>
     </row>
   </sheetData>
@@ -1178,7 +1178,7 @@
         <v>2562</v>
       </c>
       <c r="AN2" s="9" t="n">
-        <v>0</v>
+        <v>2288</v>
       </c>
       <c r="AO2" s="9" t="n">
         <v>0</v>
@@ -1341,7 +1341,7 @@
         <v>1472</v>
       </c>
       <c r="AN3" s="10" t="n">
-        <v>0</v>
+        <v>1442</v>
       </c>
       <c r="AO3" s="10" t="n">
         <v>0</v>
@@ -1504,7 +1504,7 @@
         <v>1708</v>
       </c>
       <c r="AN4" s="11" t="n">
-        <v>0</v>
+        <v>1441</v>
       </c>
       <c r="AO4" s="11" t="n">
         <v>0</v>
@@ -1667,7 +1667,7 @@
         <v>5742</v>
       </c>
       <c r="AN5" s="12" t="n">
-        <v>0</v>
+        <v>5171</v>
       </c>
       <c r="AO5" s="12" t="n">
         <v>0</v>
@@ -2166,7 +2166,7 @@
         <v>4622</v>
       </c>
       <c r="AN2" s="9" t="n">
-        <v>0</v>
+        <v>3964</v>
       </c>
       <c r="AO2" s="9" t="n">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>3456</v>
       </c>
       <c r="AN3" s="10" t="n">
-        <v>0</v>
+        <v>2586</v>
       </c>
       <c r="AO3" s="10" t="n">
         <v>0</v>
@@ -2492,7 +2492,7 @@
         <v>3475</v>
       </c>
       <c r="AN4" s="11" t="n">
-        <v>0</v>
+        <v>3062</v>
       </c>
       <c r="AO4" s="11" t="n">
         <v>0</v>
@@ -2655,7 +2655,7 @@
         <v>11553</v>
       </c>
       <c r="AN5" s="12" t="n">
-        <v>0</v>
+        <v>9612</v>
       </c>
       <c r="AO5" s="12" t="n">
         <v>0</v>
@@ -3474,16 +3474,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>2288</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>1442</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>1441</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>5171</v>
       </c>
     </row>
     <row r="41">
@@ -4510,16 +4510,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>3964</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>2586</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>3062</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>9612</v>
       </c>
     </row>
     <row r="41">
@@ -6026,16 +6026,16 @@
         <v>5132</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>2288</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>1442</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1441</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>5171</v>
       </c>
     </row>
     <row r="41">
@@ -6502,7 +6502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6974,6 +6974,18 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>C:\TRC\trc_engine\outputs\weekly\Weekly W38-2026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>W39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>C:\TRC\trc_engine\outputs\weekly\Weekly W39-2026.xlsx</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8354,7 @@
         <v>2562</v>
       </c>
       <c r="AO9" s="7" t="n">
-        <v>0</v>
+        <v>2288</v>
       </c>
       <c r="AP9" s="7" t="n">
         <v>0</v>
@@ -8510,7 +8522,7 @@
         <v>1472</v>
       </c>
       <c r="AO10" s="7" t="n">
-        <v>0</v>
+        <v>1442</v>
       </c>
       <c r="AP10" s="7" t="n">
         <v>0</v>
@@ -8678,7 +8690,7 @@
         <v>1708</v>
       </c>
       <c r="AO11" s="7" t="n">
-        <v>0</v>
+        <v>1441</v>
       </c>
       <c r="AP11" s="7" t="n">
         <v>0</v>
@@ -9178,7 +9190,7 @@
         <v>4622</v>
       </c>
       <c r="AO15" s="7" t="n">
-        <v>0</v>
+        <v>3964</v>
       </c>
       <c r="AP15" s="7" t="n">
         <v>0</v>
@@ -9346,7 +9358,7 @@
         <v>3456</v>
       </c>
       <c r="AO16" s="7" t="n">
-        <v>0</v>
+        <v>2586</v>
       </c>
       <c r="AP16" s="7" t="n">
         <v>0</v>
@@ -9514,7 +9526,7 @@
         <v>3475</v>
       </c>
       <c r="AO17" s="7" t="n">
-        <v>0</v>
+        <v>3062</v>
       </c>
       <c r="AP17" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Data export W40-2026 (2026-10-06T19:28:48Z)
</commit_message>
<xml_diff>
--- a/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
+++ b/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
@@ -643,22 +643,22 @@
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>101379</v>
+        <v>103302</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>44.40293277737872</v>
+        <v>44.31850358230726</v>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>189238:00:00</t>
+          <t>192826:00:00</t>
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>189238</v>
+        <v>192826</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>44.58197478278897</v>
+        <v>44.45904693393834</v>
       </c>
     </row>
     <row r="3">
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>58397</v>
+        <v>59718</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>25.57727009933601</v>
+        <v>25.6201467244412</v>
       </c>
       <c r="E3" s="10" t="inlineStr"/>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>109949:00:00</t>
+          <t>112595:00:00</t>
         </is>
       </c>
       <c r="G3" s="10" t="n">
-        <v>109949</v>
+        <v>112595</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>25.9025330292693</v>
+        <v>25.96053638786672</v>
       </c>
     </row>
     <row r="4">
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>68540</v>
+        <v>70070</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>30.01979712328527</v>
+        <v>30.06134969325153</v>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>125285:00:00</t>
+          <t>128295:00:00</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>125285</v>
+        <v>128295</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>29.51549218794173</v>
+        <v>29.58041667819495</v>
       </c>
     </row>
   </sheetData>
@@ -1181,7 +1181,7 @@
         <v>2288</v>
       </c>
       <c r="AO2" s="9" t="n">
-        <v>0</v>
+        <v>1923</v>
       </c>
       <c r="AP2" s="9" t="n">
         <v>0</v>
@@ -1344,7 +1344,7 @@
         <v>1442</v>
       </c>
       <c r="AO3" s="10" t="n">
-        <v>0</v>
+        <v>1321</v>
       </c>
       <c r="AP3" s="10" t="n">
         <v>0</v>
@@ -1507,7 +1507,7 @@
         <v>1441</v>
       </c>
       <c r="AO4" s="11" t="n">
-        <v>0</v>
+        <v>1530</v>
       </c>
       <c r="AP4" s="11" t="n">
         <v>0</v>
@@ -1670,7 +1670,7 @@
         <v>5171</v>
       </c>
       <c r="AO5" s="12" t="n">
-        <v>0</v>
+        <v>4774</v>
       </c>
       <c r="AP5" s="12" t="n">
         <v>0</v>
@@ -2169,7 +2169,7 @@
         <v>3964</v>
       </c>
       <c r="AO2" s="9" t="n">
-        <v>0</v>
+        <v>3588</v>
       </c>
       <c r="AP2" s="9" t="n">
         <v>0</v>
@@ -2332,7 +2332,7 @@
         <v>2586</v>
       </c>
       <c r="AO3" s="10" t="n">
-        <v>0</v>
+        <v>2646</v>
       </c>
       <c r="AP3" s="10" t="n">
         <v>0</v>
@@ -2495,7 +2495,7 @@
         <v>3062</v>
       </c>
       <c r="AO4" s="11" t="n">
-        <v>0</v>
+        <v>3010</v>
       </c>
       <c r="AP4" s="11" t="n">
         <v>0</v>
@@ -2658,7 +2658,7 @@
         <v>9612</v>
       </c>
       <c r="AO5" s="12" t="n">
-        <v>0</v>
+        <v>9244</v>
       </c>
       <c r="AP5" s="12" t="n">
         <v>0</v>
@@ -3493,16 +3493,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>1923</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>1321</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1530</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>4774</v>
       </c>
     </row>
     <row r="42">
@@ -4529,16 +4529,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>3588</v>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>2646</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>3010</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>9244</v>
       </c>
     </row>
     <row r="42">
@@ -6057,16 +6057,16 @@
         <v>5673</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>1923</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>1321</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>1530</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>4774</v>
       </c>
     </row>
     <row r="42">
@@ -6502,7 +6502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6986,6 +6986,18 @@
       <c r="B40" t="inlineStr">
         <is>
           <t>C:\TRC\trc_engine\outputs\weekly\Weekly W39-2026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>C:\TRC\trc_engine\outputs\weekly\Weekly W40-2026.xlsx</t>
         </is>
       </c>
     </row>
@@ -8357,7 +8369,7 @@
         <v>2288</v>
       </c>
       <c r="AP9" s="7" t="n">
-        <v>0</v>
+        <v>1923</v>
       </c>
       <c r="AQ9" s="7" t="n">
         <v>0</v>
@@ -8525,7 +8537,7 @@
         <v>1442</v>
       </c>
       <c r="AP10" s="7" t="n">
-        <v>0</v>
+        <v>1321</v>
       </c>
       <c r="AQ10" s="7" t="n">
         <v>0</v>
@@ -8693,7 +8705,7 @@
         <v>1441</v>
       </c>
       <c r="AP11" s="7" t="n">
-        <v>0</v>
+        <v>1530</v>
       </c>
       <c r="AQ11" s="7" t="n">
         <v>0</v>
@@ -9193,7 +9205,7 @@
         <v>3964</v>
       </c>
       <c r="AP15" s="7" t="n">
-        <v>0</v>
+        <v>3588</v>
       </c>
       <c r="AQ15" s="7" t="n">
         <v>0</v>
@@ -9361,7 +9373,7 @@
         <v>2586</v>
       </c>
       <c r="AP16" s="7" t="n">
-        <v>0</v>
+        <v>2646</v>
       </c>
       <c r="AQ16" s="7" t="n">
         <v>0</v>
@@ -9529,7 +9541,7 @@
         <v>3062</v>
       </c>
       <c r="AP17" s="7" t="n">
-        <v>0</v>
+        <v>3010</v>
       </c>
       <c r="AQ17" s="7" t="n">
         <v>0</v>

</xml_diff>